<commit_message>
Publication build from f58147510c98875659007ec285d57ba6d464d600 (v0.1.0)
</commit_message>
<xml_diff>
--- a/publication/web-root/matchsync-donor/0.1.0/StructureDefinition-nmdp-donor-patient.xlsx
+++ b/publication/web-root/matchsync-donor/0.1.0/StructureDefinition-nmdp-donor-patient.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-03T16:43:13+00:00</t>
+    <t>2026-09-22T13:14:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -849,7 +849,7 @@
     <t>NMDP GRID (Global Registration Identifier for Donors)</t>
   </si>
   <si>
-    <t>The NMDP GRID identifier that uniquely identifies a donor. A 32-character uppercase alphanumeric string (0-9 and A-F, no dashes or spaces), e.g. 99D0BA02660443B585D525525EB3F2D2. System: http://nmdp.org/identifier/grid</t>
+    <t>The NMDP GRID identifier that uniquely identifies a donor. A 19-character ISBT 128 identifier composed of a 4-digit Issuing Organization Number (ION), a donor registration number, and check characters, e.g. 6939DKM001392612726. System: http://nmdp.org/identifier/grid</t>
   </si>
   <si>
     <t>Patient.identifier:grid.id</t>

</xml_diff>